<commit_message>
feat: make acquired_date optional, align import/export headers with asset fields, update header subtitle to CMU Library
</commit_message>
<xml_diff>
--- a/public/sample_assets_import.xlsx
+++ b/public/sample_assets_import.xlsx
@@ -397,38 +397,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:P5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>asset_code</v>
+        <v>เลขครุภัณฑ์</v>
       </c>
       <c r="B1" t="str">
-        <v>name</v>
+        <v>ชื่อครุภัณฑ์</v>
       </c>
       <c r="C1" t="str">
-        <v>category_code</v>
+        <v>หมวดหมู่ครุภัณฑ์</v>
       </c>
       <c r="D1" t="str">
-        <v>department_code</v>
+        <v>สถานะครุภัณฑ์</v>
       </c>
       <c r="E1" t="str">
-        <v>brand</v>
+        <v>ยี่ห้อ (Brand)</v>
       </c>
       <c r="F1" t="str">
-        <v>model</v>
+        <v>รุ่น (Model)</v>
       </c>
       <c r="G1" t="str">
-        <v>serial_number</v>
+        <v>หมายเลขเครื่อง (Serial Number)</v>
       </c>
       <c r="H1" t="str">
-        <v>unit_price</v>
+        <v>ราคาต่อหน่วย (บาท)</v>
       </c>
       <c r="I1" t="str">
-        <v>acquired_date</v>
+        <v>วันที่รับเข้า / วันที่ตรวจรับ</v>
       </c>
       <c r="J1" t="str">
-        <v>contract_number</v>
+        <v>เลขที่สัญญาจัดซื้อ / ใบตรวจรับ</v>
+      </c>
+      <c r="K1" t="str">
+        <v>หน่วยงาน/กองผู้ครอบครอง</v>
+      </c>
+      <c r="L1" t="str">
+        <v>อาคาร / ห้อง / สถานที่ตั้ง</v>
+      </c>
+      <c r="M1" t="str">
+        <v>ผู้รับผิดชอบดูแลครุภัณฑ์</v>
+      </c>
+      <c r="N1" t="str">
+        <v>อายุการใช้งานโดยประมาณ (ปี)</v>
+      </c>
+      <c r="O1" t="str">
+        <v>คุณลักษณะเฉพาะ / รายละเอียด</v>
+      </c>
+      <c r="P1" t="str">
+        <v>หมายเหตุ</v>
       </c>
     </row>
     <row r="2">
@@ -442,7 +460,7 @@
         <v>7440</v>
       </c>
       <c r="D2" t="str">
-        <v>ITD</v>
+        <v>พร้อมใช้งาน</v>
       </c>
       <c r="E2" t="str">
         <v>Dell</v>
@@ -461,6 +479,24 @@
       </c>
       <c r="J2" t="str">
         <v>สญ.021/2569</v>
+      </c>
+      <c r="K2" t="str">
+        <v>ITD</v>
+      </c>
+      <c r="L2" t="str">
+        <v>BLD-A-405</v>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2">
+        <v>5</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Intel Core i7, RAM 16GB, SSD 512GB</v>
+      </c>
+      <c r="P2" t="str">
+        <v>ครุภัณฑ์ประจำศูนย์เทคโนโลยีสารสนเทศ</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +510,7 @@
         <v>7440</v>
       </c>
       <c r="D3" t="str">
-        <v>ADM</v>
+        <v>พร้อมใช้งาน</v>
       </c>
       <c r="E3" t="str">
         <v>HP</v>
@@ -489,10 +525,28 @@
         <v>19800</v>
       </c>
       <c r="I3" t="str">
-        <v>2026-10-16</v>
+        <v/>
       </c>
       <c r="J3" t="str">
         <v>สญ.021/2569</v>
+      </c>
+      <c r="K3" t="str">
+        <v>FAD</v>
+      </c>
+      <c r="L3" t="str">
+        <v>BLD-A-201</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3">
+        <v>5</v>
+      </c>
+      <c r="O3" t="str">
+        <v>พิมพ์สีสองหน้าอัตโนมัติ รองรับระบบเครือข่าย LAN</v>
+      </c>
+      <c r="P3" t="str">
+        <v>ใช้งานส่วนกลางกลุ่มงานบริหารพัสดุ</v>
       </c>
     </row>
     <row r="4">
@@ -506,7 +560,7 @@
         <v>7110</v>
       </c>
       <c r="D4" t="str">
-        <v>FIN</v>
+        <v>พร้อมใช้งาน</v>
       </c>
       <c r="E4" t="str">
         <v>Modernform</v>
@@ -521,10 +575,28 @@
         <v>8900</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-10-18</v>
+        <v/>
       </c>
       <c r="J4" t="str">
         <v>สญ.022/2569</v>
+      </c>
+      <c r="K4" t="str">
+        <v>GAD</v>
+      </c>
+      <c r="L4" t="str">
+        <v>BLD-B-102</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4">
+        <v>5</v>
+      </c>
+      <c r="O4" t="str">
+        <v>ขนาด 150x75x75 ซม. โครงเหล็กหน้าไม้เมลามีน</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -538,7 +610,7 @@
         <v>7730</v>
       </c>
       <c r="D5" t="str">
-        <v>PLN</v>
+        <v>พร้อมใช้งาน</v>
       </c>
       <c r="E5" t="str">
         <v>Epson</v>
@@ -557,11 +629,29 @@
       </c>
       <c r="J5" t="str">
         <v>สญ.025/2569</v>
+      </c>
+      <c r="K5" t="str">
+        <v>PLD</v>
+      </c>
+      <c r="L5" t="str">
+        <v>BLD-A-302</v>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5">
+        <v>5</v>
+      </c>
+      <c r="O5" t="str">
+        <v>ความสว่าง 5,200 Lumens ความละเอียด WUXGA</v>
+      </c>
+      <c r="P5" t="str">
+        <v>ติดตั้งประจำห้องประชุม</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 15-min session timeout, Buddhist Era (พ.ศ.) date inputs & formatting, and PANTONE color palette
</commit_message>
<xml_diff>
--- a/public/sample_assets_import.xlsx
+++ b/public/sample_assets_import.xlsx
@@ -475,7 +475,7 @@
         <v>28500</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-10-15</v>
+        <v>15/10/2569</v>
       </c>
       <c r="J2" t="str">
         <v>สญ.021/2569</v>
@@ -625,7 +625,7 @@
         <v>64000</v>
       </c>
       <c r="I5" t="str">
-        <v>2026-10-20</v>
+        <v>20/10/2569</v>
       </c>
       <c r="J5" t="str">
         <v>สญ.025/2569</v>

</xml_diff>